<commit_message>
feat: mostrar todas las estadisticas de un jugador (en progreso)
Ahora se muestran los esquemas usados como director tecnico
</commit_message>
<xml_diff>
--- a/backend/src/db/Once_Historico.xlsx
+++ b/backend/src/db/Once_Historico.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\victo\Documents\GitHub\Brumario\backend\src\db\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E898D4D6-32AE-479E-9C74-17BE302477ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6157992E-5477-4C6E-BDBF-FAF83D22E829}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C664D07F-D089-4B67-8734-91CC2386005C}"/>
   </bookViews>
@@ -1835,9 +1835,6 @@
     <t>Ubicacion</t>
   </si>
   <si>
-    <t>Esquema tactico</t>
-  </si>
-  <si>
     <t>Director Tecnico</t>
   </si>
   <si>
@@ -1971,6 +1968,9 @@
   </si>
   <si>
     <t>Empatado</t>
+  </si>
+  <si>
+    <t>Esquema Tactico</t>
   </si>
 </sst>
 </file>
@@ -2535,7 +2535,7 @@
         <v>3</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="G1" s="4" t="s">
         <v>597</v>
@@ -2559,13 +2559,13 @@
         <v>8</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="O1" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="P1" s="6" t="s">
         <v>599</v>
-      </c>
-      <c r="P1" s="6" t="s">
-        <v>600</v>
       </c>
       <c r="Q1" s="6" t="s">
         <v>9</v>
@@ -2601,49 +2601,49 @@
         <v>19</v>
       </c>
       <c r="AB1" s="6" t="s">
+        <v>625</v>
+      </c>
+      <c r="AC1" s="6" t="s">
         <v>626</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>627</v>
       </c>
-      <c r="AD1" s="6" t="s">
+      <c r="AE1" s="6" t="s">
         <v>628</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AF1" s="6" t="s">
         <v>629</v>
       </c>
-      <c r="AF1" s="6" t="s">
+      <c r="AG1" s="6" t="s">
         <v>630</v>
       </c>
-      <c r="AG1" s="6" t="s">
+      <c r="AH1" s="6" t="s">
         <v>631</v>
       </c>
-      <c r="AH1" s="6" t="s">
+      <c r="AI1" s="6" t="s">
         <v>632</v>
       </c>
-      <c r="AI1" s="6" t="s">
+      <c r="AJ1" s="6" t="s">
         <v>633</v>
       </c>
-      <c r="AJ1" s="6" t="s">
+      <c r="AK1" s="6" t="s">
         <v>634</v>
       </c>
-      <c r="AK1" s="6" t="s">
+      <c r="AL1" s="6" t="s">
         <v>635</v>
       </c>
-      <c r="AL1" s="6" t="s">
+      <c r="AM1" s="6" t="s">
         <v>636</v>
       </c>
-      <c r="AM1" s="6" t="s">
+      <c r="AN1" s="6" t="s">
         <v>637</v>
       </c>
-      <c r="AN1" s="6" t="s">
+      <c r="AO1" s="6" t="s">
         <v>638</v>
       </c>
-      <c r="AO1" s="6" t="s">
+      <c r="AP1" s="6" t="s">
         <v>639</v>
-      </c>
-      <c r="AP1" s="6" t="s">
-        <v>640</v>
       </c>
       <c r="AQ1" s="6" t="s">
         <v>20</v>
@@ -2901,7 +2901,7 @@
         <v>0</v>
       </c>
       <c r="N2" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O2" s="13"/>
       <c r="P2" s="14"/>
@@ -3035,7 +3035,7 @@
         <v>3</v>
       </c>
       <c r="N3" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O3" s="13" t="s">
         <v>104</v>
@@ -3199,7 +3199,7 @@
         <v>0</v>
       </c>
       <c r="N4" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O4" s="13" t="s">
         <v>122</v>
@@ -3357,7 +3357,7 @@
         <v>2</v>
       </c>
       <c r="N5" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O5" s="13" t="s">
         <v>122</v>
@@ -3513,7 +3513,7 @@
         <v>0</v>
       </c>
       <c r="N6" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O6" s="13" t="s">
         <v>122</v>
@@ -3669,7 +3669,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O7" s="13" t="s">
         <v>122</v>
@@ -3815,7 +3815,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O8" s="13" t="s">
         <v>122</v>
@@ -3957,7 +3957,7 @@
         <v>3</v>
       </c>
       <c r="N9" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O9" s="13" t="s">
         <v>122</v>
@@ -4115,7 +4115,7 @@
         <v>0</v>
       </c>
       <c r="N10" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O10" s="13"/>
       <c r="P10" s="14"/>
@@ -4249,7 +4249,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O11" s="13" t="s">
         <v>122</v>
@@ -4419,7 +4419,7 @@
         <v>2</v>
       </c>
       <c r="N12" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O12" s="13" t="s">
         <v>122</v>
@@ -4603,7 +4603,7 @@
         <v>2</v>
       </c>
       <c r="N13" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O13" s="13" t="s">
         <v>122</v>
@@ -4791,7 +4791,7 @@
         <v>1</v>
       </c>
       <c r="N14" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O14" s="13" t="s">
         <v>122</v>
@@ -4963,7 +4963,7 @@
         <v>1</v>
       </c>
       <c r="N15" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O15" s="13" t="s">
         <v>122</v>
@@ -5161,7 +5161,7 @@
         <v>2</v>
       </c>
       <c r="N16" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O16" s="13" t="s">
         <v>122</v>
@@ -5343,7 +5343,7 @@
         <v>1</v>
       </c>
       <c r="N17" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O17" s="13" t="s">
         <v>122</v>
@@ -5521,7 +5521,7 @@
         <v>1</v>
       </c>
       <c r="N18" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O18" s="13" t="s">
         <v>122</v>
@@ -5705,7 +5705,7 @@
         <v>1</v>
       </c>
       <c r="N19" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O19" s="13" t="s">
         <v>122</v>
@@ -5893,7 +5893,7 @@
         <v>0</v>
       </c>
       <c r="N20" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O20" s="13"/>
       <c r="P20" s="14"/>
@@ -6027,7 +6027,7 @@
         <v>0</v>
       </c>
       <c r="N21" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O21" s="13" t="s">
         <v>122</v>
@@ -6197,7 +6197,7 @@
         <v>3</v>
       </c>
       <c r="N22" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O22" s="13" t="s">
         <v>122</v>
@@ -6393,7 +6393,7 @@
         <v>0</v>
       </c>
       <c r="N23" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O23" s="13" t="s">
         <v>122</v>
@@ -6565,7 +6565,7 @@
         <v>1</v>
       </c>
       <c r="N24" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O24" s="13" t="s">
         <v>122</v>
@@ -6745,7 +6745,7 @@
         <v>0</v>
       </c>
       <c r="N25" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O25" s="13"/>
       <c r="P25" s="14"/>
@@ -6879,7 +6879,7 @@
         <v>0</v>
       </c>
       <c r="N26" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O26" s="13" t="s">
         <v>122</v>
@@ -7061,7 +7061,7 @@
         <v>7</v>
       </c>
       <c r="N27" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O27" s="15" t="s">
         <v>122</v>
@@ -7233,7 +7233,7 @@
         <v>0</v>
       </c>
       <c r="N28" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O28" s="15" t="s">
         <v>122</v>
@@ -7411,7 +7411,7 @@
         <v>1</v>
       </c>
       <c r="N29" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O29" s="15" t="s">
         <v>122</v>
@@ -7593,7 +7593,7 @@
         <v>3</v>
       </c>
       <c r="N30" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O30" s="20" t="s">
         <v>122</v>
@@ -7779,7 +7779,7 @@
         <v>0</v>
       </c>
       <c r="N31" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O31" s="20" t="s">
         <v>122</v>
@@ -7967,7 +7967,7 @@
         <v>0</v>
       </c>
       <c r="N32" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O32" s="20" t="s">
         <v>122</v>
@@ -8147,7 +8147,7 @@
         <v>1</v>
       </c>
       <c r="N33" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O33" s="20" t="s">
         <v>122</v>
@@ -8343,7 +8343,7 @@
         <v>1</v>
       </c>
       <c r="N34" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O34" s="20" t="s">
         <v>122</v>
@@ -8519,7 +8519,7 @@
         <v>2</v>
       </c>
       <c r="N35" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O35" s="20" t="s">
         <v>122</v>
@@ -8693,7 +8693,7 @@
         <v>2</v>
       </c>
       <c r="N36" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O36" s="20" t="s">
         <v>122</v>
@@ -8889,7 +8889,7 @@
         <v>2</v>
       </c>
       <c r="N37" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O37" s="20" t="s">
         <v>122</v>
@@ -9083,7 +9083,7 @@
         <v>1</v>
       </c>
       <c r="N38" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O38" s="20" t="s">
         <v>122</v>
@@ -9277,7 +9277,7 @@
         <v>0</v>
       </c>
       <c r="N39" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O39" s="20" t="s">
         <v>122</v>
@@ -9459,7 +9459,7 @@
         <v>1</v>
       </c>
       <c r="N40" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O40" s="20" t="s">
         <v>122</v>
@@ -9647,7 +9647,7 @@
         <v>2</v>
       </c>
       <c r="N41" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O41" s="20" t="s">
         <v>122</v>
@@ -9833,7 +9833,7 @@
         <v>1</v>
       </c>
       <c r="N42" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O42" s="20" t="s">
         <v>122</v>
@@ -10013,7 +10013,7 @@
         <v>1</v>
       </c>
       <c r="N43" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O43" s="20" t="s">
         <v>122</v>
@@ -10223,7 +10223,7 @@
         <v>0</v>
       </c>
       <c r="N44" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O44" s="20" t="s">
         <v>122</v>
@@ -10411,7 +10411,7 @@
         <v>3</v>
       </c>
       <c r="N45" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O45" s="20" t="s">
         <v>122</v>
@@ -10597,7 +10597,7 @@
         <v>2</v>
       </c>
       <c r="N46" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O46" s="20" t="s">
         <v>122</v>
@@ -12315,7 +12315,7 @@
         <v>0</v>
       </c>
       <c r="N55" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O55" s="15" t="s">
         <v>122</v>
@@ -12483,7 +12483,7 @@
         <v>0</v>
       </c>
       <c r="N56" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O56" s="15" t="s">
         <v>222</v>
@@ -12525,7 +12525,7 @@
         <v>114</v>
       </c>
       <c r="AB56" s="14" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="AC56" s="14" t="s">
         <v>170</v>
@@ -12717,7 +12717,7 @@
         <v>2</v>
       </c>
       <c r="N57" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O57" s="15" t="s">
         <v>222</v>
@@ -12883,7 +12883,7 @@
         <v>2</v>
       </c>
       <c r="N58" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O58" s="20" t="s">
         <v>122</v>
@@ -13061,7 +13061,7 @@
         <v>6</v>
       </c>
       <c r="N59" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O59" s="20" t="s">
         <v>122</v>
@@ -13235,7 +13235,7 @@
         <v>0</v>
       </c>
       <c r="N60" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O60" s="20" t="s">
         <v>122</v>
@@ -13425,7 +13425,7 @@
         <v>3</v>
       </c>
       <c r="N61" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O61" s="20" t="s">
         <v>122</v>
@@ -13603,7 +13603,7 @@
         <v>4</v>
       </c>
       <c r="N62" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O62" s="20" t="s">
         <v>122</v>
@@ -13789,7 +13789,7 @@
         <v>1</v>
       </c>
       <c r="N63" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O63" s="20" t="s">
         <v>122</v>
@@ -13975,7 +13975,7 @@
         <v>3</v>
       </c>
       <c r="N64" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O64" s="20" t="s">
         <v>122</v>
@@ -14159,7 +14159,7 @@
         <v>1</v>
       </c>
       <c r="N65" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O65" s="20" t="s">
         <v>240</v>
@@ -14508,7 +14508,7 @@
         <v>0</v>
       </c>
       <c r="N67" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O67" s="20" t="s">
         <v>122</v>
@@ -14694,7 +14694,7 @@
         <v>2</v>
       </c>
       <c r="N68" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O68" s="20" t="s">
         <v>122</v>
@@ -14886,7 +14886,7 @@
         <v>1</v>
       </c>
       <c r="N69" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O69" s="20" t="s">
         <v>244</v>
@@ -15080,7 +15080,7 @@
         <v>2</v>
       </c>
       <c r="N70" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O70" s="20" t="s">
         <v>247</v>
@@ -15262,7 +15262,7 @@
         <v>3</v>
       </c>
       <c r="N71" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O71" s="20" t="s">
         <v>244</v>
@@ -15440,7 +15440,7 @@
         <v>4</v>
       </c>
       <c r="N72" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O72" s="20" t="s">
         <v>122</v>
@@ -15636,7 +15636,7 @@
         <v>1</v>
       </c>
       <c r="N73" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O73" s="20" t="s">
         <v>122</v>
@@ -15836,7 +15836,7 @@
         <v>1</v>
       </c>
       <c r="N74" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O74" s="20" t="s">
         <v>250</v>
@@ -16026,7 +16026,7 @@
         <v>2</v>
       </c>
       <c r="N75" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O75" s="20" t="s">
         <v>250</v>
@@ -16214,7 +16214,7 @@
         <v>0</v>
       </c>
       <c r="N76" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O76" s="20" t="s">
         <v>122</v>
@@ -16394,7 +16394,7 @@
         <v>0</v>
       </c>
       <c r="N77" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O77" s="20" t="s">
         <v>122</v>
@@ -16608,7 +16608,7 @@
         <v>1</v>
       </c>
       <c r="N78" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O78" s="20" t="s">
         <v>122</v>
@@ -16788,7 +16788,7 @@
         <v>1</v>
       </c>
       <c r="N79" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O79" s="20" t="s">
         <v>122</v>
@@ -16978,7 +16978,7 @@
         <v>1</v>
       </c>
       <c r="N80" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O80" s="20" t="s">
         <v>122</v>
@@ -17196,7 +17196,7 @@
         <v>0</v>
       </c>
       <c r="N81" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O81" s="20" t="s">
         <v>122</v>
@@ -17384,7 +17384,7 @@
         <v>0</v>
       </c>
       <c r="N82" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O82" s="20" t="s">
         <v>122</v>
@@ -17572,7 +17572,7 @@
         <v>0</v>
       </c>
       <c r="N83" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O83" s="20" t="s">
         <v>122</v>
@@ -17762,7 +17762,7 @@
         <v>0</v>
       </c>
       <c r="N84" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O84" s="13"/>
       <c r="P84" s="14"/>
@@ -17894,7 +17894,7 @@
         <v>0</v>
       </c>
       <c r="N85" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O85" s="15" t="s">
         <v>122</v>
@@ -18054,7 +18054,7 @@
         <v>1</v>
       </c>
       <c r="N86" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O86" s="15" t="s">
         <v>122</v>
@@ -18242,7 +18242,7 @@
         <v>2</v>
       </c>
       <c r="N87" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O87" s="15" t="s">
         <v>122</v>
@@ -18426,7 +18426,7 @@
         <v>2</v>
       </c>
       <c r="N88" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O88" s="20" t="s">
         <v>122</v>
@@ -18596,7 +18596,7 @@
         <v>1</v>
       </c>
       <c r="N89" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O89" s="20" t="s">
         <v>250</v>
@@ -18788,7 +18788,7 @@
         <v>0</v>
       </c>
       <c r="N90" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O90" s="20" t="s">
         <v>264</v>
@@ -18966,7 +18966,7 @@
         <v>4</v>
       </c>
       <c r="N91" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O91" s="20" t="s">
         <v>122</v>
@@ -19134,7 +19134,7 @@
         <v>1</v>
       </c>
       <c r="N92" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O92" s="20" t="s">
         <v>122</v>
@@ -19316,7 +19316,7 @@
         <v>2</v>
       </c>
       <c r="N93" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O93" s="20" t="s">
         <v>122</v>
@@ -19500,7 +19500,7 @@
         <v>2</v>
       </c>
       <c r="N94" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O94" s="20" t="s">
         <v>250</v>
@@ -19688,7 +19688,7 @@
         <v>269</v>
       </c>
       <c r="N95" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O95" s="20" t="s">
         <v>250</v>
@@ -19860,7 +19860,7 @@
         <v>1</v>
       </c>
       <c r="N96" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O96" s="20" t="s">
         <v>122</v>
@@ -20058,7 +20058,7 @@
         <v>0</v>
       </c>
       <c r="N97" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O97" s="20" t="s">
         <v>122</v>
@@ -20588,7 +20588,7 @@
         <v>1</v>
       </c>
       <c r="N100" s="14" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O100" s="20" t="s">
         <v>122</v>
@@ -20782,7 +20782,7 @@
         <v>3</v>
       </c>
       <c r="N101" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O101" s="20" t="s">
         <v>122</v>
@@ -20988,7 +20988,7 @@
         <v>1</v>
       </c>
       <c r="N102" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O102" s="20" t="s">
         <v>122</v>
@@ -21170,7 +21170,7 @@
         <v>0</v>
       </c>
       <c r="N103" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O103" s="20" t="s">
         <v>122</v>
@@ -21370,7 +21370,7 @@
         <v>2</v>
       </c>
       <c r="N104" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O104" s="20" t="s">
         <v>122</v>
@@ -21560,7 +21560,7 @@
         <v>1</v>
       </c>
       <c r="N105" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O105" s="20" t="s">
         <v>122</v>
@@ -21746,7 +21746,7 @@
         <v>0</v>
       </c>
       <c r="N106" s="12" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O106" s="20" t="s">
         <v>122</v>
@@ -21916,7 +21916,7 @@
         <v>1</v>
       </c>
       <c r="N107" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O107" s="20" t="s">
         <v>122</v>
@@ -22110,7 +22110,7 @@
         <v>2</v>
       </c>
       <c r="N108" s="12" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O108" s="20" t="s">
         <v>279</v>
@@ -22276,7 +22276,7 @@
         <v>1</v>
       </c>
       <c r="N109" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O109" s="20" t="s">
         <v>122</v>
@@ -22456,7 +22456,7 @@
         <v>1</v>
       </c>
       <c r="N110" s="12" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O110" s="15" t="s">
         <v>284</v>
@@ -22634,7 +22634,7 @@
         <v>1</v>
       </c>
       <c r="N111" s="18" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O111" s="15" t="s">
         <v>279</v>
@@ -22804,7 +22804,7 @@
         <v>0</v>
       </c>
       <c r="N112" s="18" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O112" s="15" t="s">
         <v>122</v>
@@ -22978,7 +22978,7 @@
         <v>4</v>
       </c>
       <c r="N113" s="18" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O113" s="15" t="s">
         <v>122</v>
@@ -23023,7 +23023,7 @@
         <v>124</v>
       </c>
       <c r="AC113" s="14" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AD113" s="14" t="s">
         <v>109</v>
@@ -23156,7 +23156,7 @@
         <v>1</v>
       </c>
       <c r="N114" s="18" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O114" s="15" t="s">
         <v>250</v>
@@ -23201,7 +23201,7 @@
         <v>139</v>
       </c>
       <c r="AC114" s="14" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="AD114" s="14" t="s">
         <v>138</v>
@@ -23328,7 +23328,7 @@
         <v>0</v>
       </c>
       <c r="N115" s="18" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O115" s="15" t="s">
         <v>122</v>
@@ -23522,7 +23522,7 @@
         <v>2</v>
       </c>
       <c r="N116" s="18" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O116" s="15" t="s">
         <v>122</v>
@@ -23720,7 +23720,7 @@
         <v>1</v>
       </c>
       <c r="N117" s="18" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O117" s="15" t="s">
         <v>122</v>
@@ -23906,7 +23906,7 @@
         <v>4</v>
       </c>
       <c r="N118" s="18" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O118" s="15" t="s">
         <v>240</v>
@@ -24082,7 +24082,7 @@
         <v>1</v>
       </c>
       <c r="N119" s="18" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O119" s="15" t="s">
         <v>122</v>
@@ -24268,7 +24268,7 @@
         <v>1</v>
       </c>
       <c r="N120" s="18" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O120" s="15" t="s">
         <v>122</v>
@@ -24452,7 +24452,7 @@
         <v>1</v>
       </c>
       <c r="N121" s="18" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O121" s="15" t="s">
         <v>122</v>
@@ -24873,7 +24873,7 @@
         <v>297</v>
       </c>
       <c r="AE123" s="14" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="AF123" s="14" t="s">
         <v>124</v>
@@ -27302,7 +27302,7 @@
         <v>191</v>
       </c>
       <c r="AC136" s="14" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="AD136" s="14" t="s">
         <v>146</v>
@@ -27708,13 +27708,13 @@
         <v>113</v>
       </c>
       <c r="AE138" s="14" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="AF138" s="14" t="s">
         <v>170</v>
       </c>
       <c r="AG138" s="14" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="AH138" s="14" t="s">
         <v>181</v>
@@ -28324,7 +28324,7 @@
         <v>316</v>
       </c>
       <c r="AH141" s="14" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="AI141" s="14"/>
       <c r="AJ141" s="14"/>
@@ -29229,7 +29229,7 @@
         <v>181</v>
       </c>
       <c r="AB146" s="14" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="AC146" s="14" t="s">
         <v>146</v>
@@ -30888,10 +30888,10 @@
         <v>297</v>
       </c>
       <c r="AF155" s="14" t="s">
+        <v>609</v>
+      </c>
+      <c r="AG155" s="14" t="s">
         <v>610</v>
-      </c>
-      <c r="AG155" s="14" t="s">
-        <v>611</v>
       </c>
       <c r="AH155" s="14" t="s">
         <v>146</v>
@@ -32701,7 +32701,7 @@
         <v>1</v>
       </c>
       <c r="N165" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O165" s="15" t="s">
         <v>122</v>
@@ -32887,7 +32887,7 @@
         <v>3</v>
       </c>
       <c r="N166" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O166" s="15" t="s">
         <v>122</v>
@@ -33053,7 +33053,7 @@
         <v>1</v>
       </c>
       <c r="N167" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O167" s="15" t="s">
         <v>122</v>
@@ -33235,7 +33235,7 @@
         <v>7</v>
       </c>
       <c r="N168" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O168" s="15" t="s">
         <v>122</v>
@@ -33419,7 +33419,7 @@
         <v>4</v>
       </c>
       <c r="N169" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O169" s="15" t="s">
         <v>250</v>
@@ -33587,7 +33587,7 @@
         <v>0</v>
       </c>
       <c r="N170" s="16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O170" s="15" t="s">
         <v>240</v>
@@ -33761,7 +33761,7 @@
         <v>5</v>
       </c>
       <c r="N171" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O171" s="15" t="s">
         <v>250</v>
@@ -33935,7 +33935,7 @@
         <v>0</v>
       </c>
       <c r="N172" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O172" s="15" t="s">
         <v>240</v>
@@ -34119,7 +34119,7 @@
         <v>1</v>
       </c>
       <c r="N173" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O173" s="15" t="s">
         <v>122</v>
@@ -34315,7 +34315,7 @@
         <v>2</v>
       </c>
       <c r="N174" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O174" s="15" t="s">
         <v>122</v>
@@ -34497,7 +34497,7 @@
         <v>4</v>
       </c>
       <c r="N175" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O175" s="15" t="s">
         <v>122</v>
@@ -34679,7 +34679,7 @@
         <v>0</v>
       </c>
       <c r="N176" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O176" s="13"/>
       <c r="P176" s="14"/>
@@ -34813,7 +34813,7 @@
         <v>2</v>
       </c>
       <c r="N177" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O177" s="15" t="s">
         <v>240</v>
@@ -34999,7 +34999,7 @@
         <v>3</v>
       </c>
       <c r="N178" s="16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O178" s="15" t="s">
         <v>240</v>
@@ -35211,7 +35211,7 @@
         <v>3</v>
       </c>
       <c r="N179" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O179" s="15" t="s">
         <v>122</v>
@@ -35401,7 +35401,7 @@
         <v>1</v>
       </c>
       <c r="N180" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O180" s="15" t="s">
         <v>122</v>
@@ -35615,7 +35615,7 @@
         <v>2</v>
       </c>
       <c r="N181" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O181" s="15" t="s">
         <v>122</v>
@@ -35793,7 +35793,7 @@
         <v>0</v>
       </c>
       <c r="N182" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O182" s="15" t="s">
         <v>122</v>
@@ -35987,7 +35987,7 @@
         <v>3</v>
       </c>
       <c r="N183" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O183" s="15" t="s">
         <v>122</v>
@@ -36145,7 +36145,7 @@
         <v>0</v>
       </c>
       <c r="N184" s="16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O184" s="15" t="s">
         <v>247</v>
@@ -36317,7 +36317,7 @@
         <v>0</v>
       </c>
       <c r="N185" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O185" s="15" t="s">
         <v>284</v>
@@ -36499,7 +36499,7 @@
         <v>2</v>
       </c>
       <c r="N186" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O186" s="15" t="s">
         <v>122</v>
@@ -36675,7 +36675,7 @@
         <v>0</v>
       </c>
       <c r="N187" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O187" s="15" t="s">
         <v>284</v>
@@ -36857,7 +36857,7 @@
         <v>1</v>
       </c>
       <c r="N188" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O188" s="15" t="s">
         <v>122</v>
@@ -37039,7 +37039,7 @@
         <v>2</v>
       </c>
       <c r="N189" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O189" s="15" t="s">
         <v>240</v>
@@ -37227,7 +37227,7 @@
         <v>0</v>
       </c>
       <c r="N190" s="16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O190" s="15" t="s">
         <v>284</v>
@@ -37403,7 +37403,7 @@
         <v>1</v>
       </c>
       <c r="N191" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O191" s="15" t="s">
         <v>284</v>
@@ -37575,7 +37575,7 @@
         <v>0</v>
       </c>
       <c r="N192" s="16" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O192" s="15" t="s">
         <v>122</v>
@@ -37747,7 +37747,7 @@
         <v>1</v>
       </c>
       <c r="N193" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O193" s="15" t="s">
         <v>122</v>
@@ -37937,7 +37937,7 @@
         <v>1</v>
       </c>
       <c r="N194" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O194" s="15" t="s">
         <v>122</v>
@@ -38123,7 +38123,7 @@
         <v>2</v>
       </c>
       <c r="N195" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O195" s="15" t="s">
         <v>284</v>
@@ -38307,7 +38307,7 @@
         <v>1</v>
       </c>
       <c r="N196" s="16" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O196" s="15" t="s">
         <v>284</v>
@@ -38477,7 +38477,7 @@
         <v>1</v>
       </c>
       <c r="N197" s="16" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O197" s="15" t="s">
         <v>122</v>
@@ -38685,7 +38685,7 @@
         <v>2</v>
       </c>
       <c r="N198" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O198" s="15" t="s">
         <v>122</v>
@@ -38863,7 +38863,7 @@
         <v>0</v>
       </c>
       <c r="N199" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O199" s="15" t="s">
         <v>122</v>
@@ -39077,7 +39077,7 @@
         <v>0</v>
       </c>
       <c r="N200" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O200" s="15" t="s">
         <v>250</v>
@@ -39293,7 +39293,7 @@
         <v>1</v>
       </c>
       <c r="N201" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O201" s="15" t="s">
         <v>122</v>
@@ -39477,7 +39477,7 @@
         <v>2</v>
       </c>
       <c r="N202" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O202" s="15" t="s">
         <v>122</v>
@@ -39691,7 +39691,7 @@
         <v>1</v>
       </c>
       <c r="N203" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O203" s="15" t="s">
         <v>122</v>
@@ -39869,7 +39869,7 @@
         <v>1</v>
       </c>
       <c r="N204" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O204" s="15" t="s">
         <v>122</v>
@@ -40075,7 +40075,7 @@
         <v>3</v>
       </c>
       <c r="N205" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O205" s="15" t="s">
         <v>122</v>
@@ -40261,7 +40261,7 @@
         <v>2</v>
       </c>
       <c r="N206" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O206" s="15" t="s">
         <v>122</v>
@@ -40447,7 +40447,7 @@
         <v>0</v>
       </c>
       <c r="N207" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O207" s="15" t="s">
         <v>122</v>
@@ -40669,7 +40669,7 @@
         <v>6</v>
       </c>
       <c r="N208" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O208" s="15" t="s">
         <v>122</v>
@@ -40711,7 +40711,7 @@
         <v>181</v>
       </c>
       <c r="AB208" s="14" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="AC208" s="14" t="s">
         <v>107</v>
@@ -40875,7 +40875,7 @@
         <v>3</v>
       </c>
       <c r="N209" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O209" s="15" t="s">
         <v>122</v>
@@ -41065,7 +41065,7 @@
         <v>1</v>
       </c>
       <c r="N210" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O210" s="15" t="s">
         <v>122</v>
@@ -41263,7 +41263,7 @@
         <v>3</v>
       </c>
       <c r="N211" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O211" s="15" t="s">
         <v>122</v>
@@ -41447,7 +41447,7 @@
         <v>2</v>
       </c>
       <c r="N212" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O212" s="15"/>
       <c r="P212" s="14"/>
@@ -41589,7 +41589,7 @@
         <v>0</v>
       </c>
       <c r="N213" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O213" s="15" t="s">
         <v>122</v>
@@ -41805,7 +41805,7 @@
         <v>3</v>
       </c>
       <c r="N214" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O214" s="15" t="s">
         <v>122</v>
@@ -41853,7 +41853,7 @@
         <v>394</v>
       </c>
       <c r="AD214" s="14" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="AE214" s="14" t="s">
         <v>370</v>
@@ -42039,7 +42039,7 @@
         <v>2</v>
       </c>
       <c r="N215" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O215" s="15" t="s">
         <v>247</v>
@@ -42237,7 +42237,7 @@
         <v>0</v>
       </c>
       <c r="N216" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O216" s="15" t="s">
         <v>413</v>
@@ -42441,7 +42441,7 @@
         <v>1</v>
       </c>
       <c r="N217" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O217" s="15" t="s">
         <v>415</v>
@@ -42639,7 +42639,7 @@
         <v>0</v>
       </c>
       <c r="N218" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O218" s="15" t="s">
         <v>122</v>
@@ -42833,7 +42833,7 @@
         <v>1</v>
       </c>
       <c r="N219" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O219" s="15" t="s">
         <v>247</v>
@@ -43029,7 +43029,7 @@
         <v>2</v>
       </c>
       <c r="N220" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O220" s="15" t="s">
         <v>418</v>
@@ -43074,13 +43074,13 @@
         <v>300</v>
       </c>
       <c r="AC220" s="14" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AD220" s="14" t="s">
         <v>297</v>
       </c>
       <c r="AE220" s="14" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="AF220" s="14" t="s">
         <v>420</v>
@@ -43213,7 +43213,7 @@
         <v>0</v>
       </c>
       <c r="N221" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O221" s="15"/>
       <c r="P221" s="14"/>
@@ -43357,7 +43357,7 @@
         <v>1</v>
       </c>
       <c r="N222" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O222" s="15" t="s">
         <v>247</v>
@@ -43545,7 +43545,7 @@
         <v>0</v>
       </c>
       <c r="N223" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O223" s="15"/>
       <c r="P223" s="14"/>
@@ -43687,7 +43687,7 @@
         <v>2</v>
       </c>
       <c r="N224" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O224" s="15" t="s">
         <v>413</v>
@@ -43873,7 +43873,7 @@
         <v>1</v>
       </c>
       <c r="N225" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O225" s="15" t="s">
         <v>247</v>
@@ -44083,7 +44083,7 @@
         <v>1</v>
       </c>
       <c r="N226" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O226" s="15" t="s">
         <v>244</v>
@@ -44125,7 +44125,7 @@
         <v>429</v>
       </c>
       <c r="AB226" s="14" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AC226" s="14" t="s">
         <v>431</v>
@@ -44273,7 +44273,7 @@
         <v>0</v>
       </c>
       <c r="N227" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O227" s="15" t="s">
         <v>415</v>
@@ -44497,7 +44497,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O228" s="15" t="s">
         <v>244</v>
@@ -44683,7 +44683,7 @@
         <v>2</v>
       </c>
       <c r="N229" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O229" s="15" t="s">
         <v>415</v>
@@ -44871,7 +44871,7 @@
         <v>0</v>
       </c>
       <c r="N230" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O230" s="15"/>
       <c r="P230" s="14"/>
@@ -45015,7 +45015,7 @@
         <v>3</v>
       </c>
       <c r="N231" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O231" s="15" t="s">
         <v>247</v>
@@ -45069,7 +45069,7 @@
         <v>429</v>
       </c>
       <c r="AF231" s="14" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="AG231" s="14"/>
       <c r="AH231" s="14"/>
@@ -45225,7 +45225,7 @@
         <v>0</v>
       </c>
       <c r="N232" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O232" s="15" t="s">
         <v>247</v>
@@ -45427,7 +45427,7 @@
         <v>0</v>
       </c>
       <c r="N233" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O233" s="15" t="s">
         <v>244</v>
@@ -45653,7 +45653,7 @@
         <v>1</v>
       </c>
       <c r="N234" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O234" s="15" t="s">
         <v>247</v>
@@ -45843,7 +45843,7 @@
         <v>2</v>
       </c>
       <c r="N235" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O235" s="15" t="s">
         <v>413</v>
@@ -46035,7 +46035,7 @@
         <v>3</v>
       </c>
       <c r="N236" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O236" s="15" t="s">
         <v>244</v>
@@ -46241,7 +46241,7 @@
         <v>0</v>
       </c>
       <c r="N237" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O237" s="15"/>
       <c r="P237" s="14"/>
@@ -46385,7 +46385,7 @@
         <v>2</v>
       </c>
       <c r="N238" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O238" s="15" t="s">
         <v>415</v>
@@ -46621,7 +46621,7 @@
         <v>0</v>
       </c>
       <c r="N239" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O239" s="15" t="s">
         <v>415</v>
@@ -46823,7 +46823,7 @@
         <v>0</v>
       </c>
       <c r="N240" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O240" s="15"/>
       <c r="P240" s="14"/>
@@ -46965,7 +46965,7 @@
         <v>4</v>
       </c>
       <c r="N241" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O241" s="15" t="s">
         <v>244</v>
@@ -47143,7 +47143,7 @@
         <v>0</v>
       </c>
       <c r="N242" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O242" s="15" t="s">
         <v>415</v>
@@ -47345,7 +47345,7 @@
         <v>0</v>
       </c>
       <c r="N243" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O243" s="15"/>
       <c r="P243" s="14"/>
@@ -47489,7 +47489,7 @@
         <v>3</v>
       </c>
       <c r="N244" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O244" s="15" t="s">
         <v>415</v>
@@ -47719,7 +47719,7 @@
         <v>1</v>
       </c>
       <c r="N245" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O245" s="15" t="s">
         <v>247</v>
@@ -47935,7 +47935,7 @@
         <v>0</v>
       </c>
       <c r="N246" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O246" s="15" t="s">
         <v>247</v>
@@ -48121,7 +48121,7 @@
         <v>1</v>
       </c>
       <c r="N247" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O247" s="15" t="s">
         <v>415</v>
@@ -48329,7 +48329,7 @@
         <v>1</v>
       </c>
       <c r="N248" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O248" s="15" t="s">
         <v>415</v>
@@ -48523,7 +48523,7 @@
         <v>3</v>
       </c>
       <c r="N249" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O249" s="15" t="s">
         <v>467</v>
@@ -48707,7 +48707,7 @@
         <v>1</v>
       </c>
       <c r="N250" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O250" s="15" t="s">
         <v>415</v>
@@ -48755,7 +48755,7 @@
         <v>471</v>
       </c>
       <c r="AD250" s="14" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AE250" s="14" t="s">
         <v>472</v>
@@ -48903,7 +48903,7 @@
         <v>0</v>
       </c>
       <c r="N251" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O251" s="15" t="s">
         <v>415</v>
@@ -48948,7 +48948,7 @@
         <v>422</v>
       </c>
       <c r="AC251" s="14" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="AD251" s="14" t="s">
         <v>300</v>
@@ -49115,7 +49115,7 @@
         <v>4</v>
       </c>
       <c r="N252" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O252" s="15" t="s">
         <v>415</v>
@@ -49157,7 +49157,7 @@
         <v>368</v>
       </c>
       <c r="AB252" s="14" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="AC252" s="14" t="s">
         <v>422</v>
@@ -49309,7 +49309,7 @@
         <v>0</v>
       </c>
       <c r="N253" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O253" s="15" t="s">
         <v>415</v>
@@ -49491,7 +49491,7 @@
         <v>3</v>
       </c>
       <c r="N254" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O254" s="15" t="s">
         <v>247</v>
@@ -49693,7 +49693,7 @@
         <v>2</v>
       </c>
       <c r="N255" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O255" s="15" t="s">
         <v>247</v>
@@ -49869,7 +49869,7 @@
         <v>1</v>
       </c>
       <c r="N256" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O256" s="15" t="s">
         <v>279</v>
@@ -50065,7 +50065,7 @@
         <v>2</v>
       </c>
       <c r="N257" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O257" s="15" t="s">
         <v>284</v>
@@ -50259,7 +50259,7 @@
         <v>2</v>
       </c>
       <c r="N258" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O258" s="15" t="s">
         <v>122</v>
@@ -50455,7 +50455,7 @@
         <v>1</v>
       </c>
       <c r="N259" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O259" s="15" t="s">
         <v>122</v>
@@ -50635,7 +50635,7 @@
         <v>2</v>
       </c>
       <c r="N260" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O260" s="15"/>
       <c r="P260" s="14"/>
@@ -50777,7 +50777,7 @@
         <v>0</v>
       </c>
       <c r="N261" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O261" s="15"/>
       <c r="P261" s="14"/>
@@ -50921,7 +50921,7 @@
         <v>2</v>
       </c>
       <c r="N262" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O262" s="15" t="s">
         <v>122</v>
@@ -51109,7 +51109,7 @@
         <v>0</v>
       </c>
       <c r="N263" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O263" s="15" t="s">
         <v>122</v>
@@ -51313,7 +51313,7 @@
         <v>0</v>
       </c>
       <c r="N264" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O264" s="15" t="s">
         <v>122</v>
@@ -51529,7 +51529,7 @@
         <v>2</v>
       </c>
       <c r="N265" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O265" s="15" t="s">
         <v>122</v>
@@ -51719,7 +51719,7 @@
         <v>1</v>
       </c>
       <c r="N266" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O266" s="15" t="s">
         <v>122</v>
@@ -51927,7 +51927,7 @@
         <v>0</v>
       </c>
       <c r="N267" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O267" s="15" t="s">
         <v>122</v>
@@ -52117,7 +52117,7 @@
         <v>0</v>
       </c>
       <c r="N268" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O268" s="15" t="s">
         <v>122</v>
@@ -52317,7 +52317,7 @@
         <v>0</v>
       </c>
       <c r="N269" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O269" s="15" t="s">
         <v>122</v>
@@ -52539,7 +52539,7 @@
         <v>2</v>
       </c>
       <c r="N270" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O270" s="15" t="s">
         <v>122</v>
@@ -52745,7 +52745,7 @@
         <v>2</v>
       </c>
       <c r="N271" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O271" s="15" t="s">
         <v>122</v>
@@ -52959,7 +52959,7 @@
         <v>2</v>
       </c>
       <c r="N272" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O272" s="15" t="s">
         <v>122</v>
@@ -53183,7 +53183,7 @@
         <v>2</v>
       </c>
       <c r="N273" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O273" s="15" t="s">
         <v>122</v>
@@ -53401,7 +53401,7 @@
         <v>2</v>
       </c>
       <c r="N274" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O274" s="15" t="s">
         <v>122</v>
@@ -53593,7 +53593,7 @@
         <v>3</v>
       </c>
       <c r="N275" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O275" s="15" t="s">
         <v>122</v>
@@ -53777,7 +53777,7 @@
         <v>0</v>
       </c>
       <c r="N276" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O276" s="15" t="s">
         <v>122</v>
@@ -53965,7 +53965,7 @@
         <v>0</v>
       </c>
       <c r="N277" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O277" s="15" t="s">
         <v>122</v>
@@ -54175,7 +54175,7 @@
         <v>0</v>
       </c>
       <c r="N278" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O278" s="15" t="s">
         <v>122</v>
@@ -54381,7 +54381,7 @@
         <v>3</v>
       </c>
       <c r="N279" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O279" s="15" t="s">
         <v>122</v>
@@ -54591,7 +54591,7 @@
         <v>0</v>
       </c>
       <c r="N280" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O280" s="15"/>
       <c r="P280" s="14"/>
@@ -54733,7 +54733,7 @@
         <v>1</v>
       </c>
       <c r="N281" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O281" s="15" t="s">
         <v>511</v>
@@ -54921,7 +54921,7 @@
         <v>1</v>
       </c>
       <c r="N282" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O282" s="15" t="s">
         <v>122</v>
@@ -55119,7 +55119,7 @@
         <v>3</v>
       </c>
       <c r="N283" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O283" s="15" t="s">
         <v>122</v>
@@ -55303,7 +55303,7 @@
         <v>2</v>
       </c>
       <c r="N284" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O284" s="15" t="s">
         <v>122</v>
@@ -55345,7 +55345,7 @@
         <v>503</v>
       </c>
       <c r="AB284" s="14" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="AC284" s="14" t="s">
         <v>112</v>
@@ -55485,7 +55485,7 @@
         <v>0</v>
       </c>
       <c r="N285" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O285" s="15" t="s">
         <v>122</v>
@@ -55681,7 +55681,7 @@
         <v>0</v>
       </c>
       <c r="N286" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O286" s="15" t="s">
         <v>122</v>
@@ -55861,7 +55861,7 @@
         <v>3</v>
       </c>
       <c r="N287" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O287" s="15" t="s">
         <v>122</v>
@@ -56037,7 +56037,7 @@
         <v>3</v>
       </c>
       <c r="N288" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O288" s="15" t="s">
         <v>122</v>
@@ -56219,7 +56219,7 @@
         <v>3</v>
       </c>
       <c r="N289" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O289" s="15" t="s">
         <v>122</v>
@@ -56413,7 +56413,7 @@
         <v>1</v>
       </c>
       <c r="N290" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O290" s="15" t="s">
         <v>122</v>
@@ -56619,7 +56619,7 @@
         <v>4</v>
       </c>
       <c r="N291" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O291" s="15" t="s">
         <v>122</v>
@@ -56795,7 +56795,7 @@
         <v>3</v>
       </c>
       <c r="N292" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O292" s="15" t="s">
         <v>250</v>
@@ -57019,7 +57019,7 @@
         <v>0</v>
       </c>
       <c r="N293" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O293" s="15"/>
       <c r="P293" s="14"/>
@@ -57163,7 +57163,7 @@
         <v>1</v>
       </c>
       <c r="N294" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O294" s="15" t="s">
         <v>122</v>
@@ -57357,7 +57357,7 @@
         <v>3</v>
       </c>
       <c r="N295" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O295" s="15" t="s">
         <v>122</v>
@@ -57547,7 +57547,7 @@
         <v>0</v>
       </c>
       <c r="N296" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O296" s="15" t="s">
         <v>122</v>
@@ -57721,7 +57721,7 @@
         <v>0</v>
       </c>
       <c r="N297" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O297" s="15"/>
       <c r="P297" s="14"/>
@@ -57865,7 +57865,7 @@
         <v>1</v>
       </c>
       <c r="N298" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O298" s="15" t="s">
         <v>122</v>
@@ -58053,7 +58053,7 @@
         <v>4</v>
       </c>
       <c r="N299" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O299" s="15" t="s">
         <v>250</v>
@@ -58239,7 +58239,7 @@
         <v>0</v>
       </c>
       <c r="N300" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O300" s="15"/>
       <c r="P300" s="14"/>
@@ -58383,7 +58383,7 @@
         <v>3</v>
       </c>
       <c r="N301" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O301" s="15" t="s">
         <v>247</v>
@@ -58573,7 +58573,7 @@
         <v>0</v>
       </c>
       <c r="N302" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O302" s="15" t="s">
         <v>279</v>
@@ -58769,7 +58769,7 @@
         <v>4</v>
       </c>
       <c r="N303" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O303" s="15" t="s">
         <v>122</v>
@@ -58967,7 +58967,7 @@
         <v>1</v>
       </c>
       <c r="N304" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O304" s="15" t="s">
         <v>247</v>
@@ -59177,7 +59177,7 @@
         <v>3</v>
       </c>
       <c r="N305" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O305" s="15" t="s">
         <v>247</v>
@@ -59381,7 +59381,7 @@
         <v>1</v>
       </c>
       <c r="N306" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O306" s="15" t="s">
         <v>250</v>
@@ -59569,7 +59569,7 @@
         <v>0</v>
       </c>
       <c r="N307" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O307" s="15" t="s">
         <v>247</v>
@@ -59747,7 +59747,7 @@
         <v>2</v>
       </c>
       <c r="N308" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O308" s="15" t="s">
         <v>247</v>
@@ -59798,7 +59798,7 @@
         <v>139</v>
       </c>
       <c r="AE308" s="14" t="s">
-        <v>620</v>
+        <v>619</v>
       </c>
       <c r="AF308" s="14" t="s">
         <v>522</v>
@@ -59931,7 +59931,7 @@
         <v>1</v>
       </c>
       <c r="N309" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O309" s="15" t="s">
         <v>528</v>
@@ -60107,7 +60107,7 @@
         <v>0</v>
       </c>
       <c r="N310" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O310" s="15"/>
       <c r="P310" s="14"/>
@@ -60251,7 +60251,7 @@
         <v>3</v>
       </c>
       <c r="N311" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O311" s="15" t="s">
         <v>247</v>
@@ -60431,7 +60431,7 @@
         <v>5</v>
       </c>
       <c r="N312" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O312" s="15" t="s">
         <v>122</v>
@@ -60613,7 +60613,7 @@
         <v>0</v>
       </c>
       <c r="N313" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O313" s="15"/>
       <c r="P313" s="14"/>
@@ -60757,7 +60757,7 @@
         <v>4</v>
       </c>
       <c r="N314" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O314" s="15" t="s">
         <v>247</v>
@@ -60931,7 +60931,7 @@
         <v>0</v>
       </c>
       <c r="N315" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O315" s="15" t="s">
         <v>122</v>
@@ -61121,7 +61121,7 @@
         <v>2</v>
       </c>
       <c r="N316" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O316" s="15" t="s">
         <v>122</v>
@@ -61319,7 +61319,7 @@
         <v>546</v>
       </c>
       <c r="N317" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O317" s="15" t="s">
         <v>122</v>
@@ -61525,7 +61525,7 @@
         <v>0</v>
       </c>
       <c r="N318" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O318" s="15" t="s">
         <v>122</v>
@@ -61765,7 +61765,7 @@
         <v>2</v>
       </c>
       <c r="N319" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O319" s="15" t="s">
         <v>122</v>
@@ -61947,7 +61947,7 @@
         <v>3</v>
       </c>
       <c r="N320" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O320" s="15" t="s">
         <v>122</v>
@@ -62125,7 +62125,7 @@
         <v>1</v>
       </c>
       <c r="N321" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O321" s="15" t="s">
         <v>122</v>
@@ -62321,7 +62321,7 @@
         <v>0</v>
       </c>
       <c r="N322" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O322" s="15" t="s">
         <v>122</v>
@@ -62541,7 +62541,7 @@
         <v>0</v>
       </c>
       <c r="N323" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O323" s="15"/>
       <c r="P323" s="14"/>
@@ -62685,7 +62685,7 @@
         <v>2</v>
       </c>
       <c r="N324" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O324" s="15" t="s">
         <v>122</v>
@@ -62893,7 +62893,7 @@
         <v>3</v>
       </c>
       <c r="N325" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O325" s="15" t="s">
         <v>122</v>
@@ -63077,7 +63077,7 @@
         <v>2</v>
       </c>
       <c r="N326" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O326" s="15" t="s">
         <v>122</v>
@@ -63269,7 +63269,7 @@
         <v>3</v>
       </c>
       <c r="N327" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O327" s="15" t="s">
         <v>122</v>
@@ -63455,7 +63455,7 @@
         <v>2</v>
       </c>
       <c r="N328" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O328" s="15" t="s">
         <v>122</v>
@@ -63647,7 +63647,7 @@
         <v>3</v>
       </c>
       <c r="N329" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O329" s="15" t="s">
         <v>415</v>
@@ -63837,7 +63837,7 @@
         <v>0</v>
       </c>
       <c r="N330" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O330" s="15"/>
       <c r="P330" s="14"/>
@@ -63979,7 +63979,7 @@
         <v>1</v>
       </c>
       <c r="N331" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O331" s="15" t="s">
         <v>247</v>
@@ -64181,7 +64181,7 @@
         <v>2</v>
       </c>
       <c r="N332" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O332" s="15"/>
       <c r="P332" s="14"/>
@@ -64323,7 +64323,7 @@
         <v>1</v>
       </c>
       <c r="N333" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O333" s="15" t="s">
         <v>528</v>
@@ -64525,7 +64525,7 @@
         <v>0</v>
       </c>
       <c r="N334" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O334" s="15" t="s">
         <v>528</v>
@@ -64573,7 +64573,7 @@
         <v>108</v>
       </c>
       <c r="AD334" s="14" t="s">
-        <v>621</v>
+        <v>620</v>
       </c>
       <c r="AE334" s="14" t="s">
         <v>112</v>
@@ -64727,7 +64727,7 @@
         <v>1</v>
       </c>
       <c r="N335" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O335" s="15" t="s">
         <v>247</v>
@@ -64933,7 +64933,7 @@
         <v>0</v>
       </c>
       <c r="N336" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O336" s="15" t="s">
         <v>528</v>
@@ -65125,7 +65125,7 @@
         <v>1</v>
       </c>
       <c r="N337" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O337" s="15" t="s">
         <v>528</v>
@@ -65321,7 +65321,7 @@
         <v>3</v>
       </c>
       <c r="N338" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O338" s="15" t="s">
         <v>528</v>
@@ -65517,7 +65517,7 @@
         <v>1</v>
       </c>
       <c r="N339" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O339" s="15" t="s">
         <v>415</v>
@@ -65562,7 +65562,7 @@
         <v>108</v>
       </c>
       <c r="AC339" s="14" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="AD339" s="14"/>
       <c r="AE339" s="14"/>
@@ -65715,7 +65715,7 @@
         <v>2</v>
       </c>
       <c r="N340" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O340" s="15" t="s">
         <v>415</v>
@@ -65909,7 +65909,7 @@
         <v>2</v>
       </c>
       <c r="N341" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O341" s="15" t="s">
         <v>572</v>
@@ -66083,7 +66083,7 @@
         <v>2</v>
       </c>
       <c r="N342" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O342" s="15" t="s">
         <v>415</v>
@@ -66303,7 +66303,7 @@
         <v>4</v>
       </c>
       <c r="N343" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O343" s="15" t="s">
         <v>244</v>
@@ -66503,7 +66503,7 @@
         <v>1</v>
       </c>
       <c r="N344" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O344" s="15" t="s">
         <v>415</v>
@@ -66701,7 +66701,7 @@
         <v>2</v>
       </c>
       <c r="N345" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O345" s="15" t="s">
         <v>415</v>
@@ -66897,7 +66897,7 @@
         <v>1</v>
       </c>
       <c r="N346" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O346" s="15" t="s">
         <v>528</v>
@@ -67099,7 +67099,7 @@
         <v>2</v>
       </c>
       <c r="N347" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O347" s="15" t="s">
         <v>528</v>
@@ -67285,7 +67285,7 @@
         <v>1</v>
       </c>
       <c r="N348" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O348" s="15" t="s">
         <v>415</v>
@@ -67473,7 +67473,7 @@
         <v>0</v>
       </c>
       <c r="N349" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O349" s="15" t="s">
         <v>415</v>
@@ -67521,7 +67521,7 @@
         <v>566</v>
       </c>
       <c r="AD349" s="14" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="AE349" s="14"/>
       <c r="AF349" s="14"/>
@@ -67675,7 +67675,7 @@
         <v>0</v>
       </c>
       <c r="N350" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O350" s="15" t="s">
         <v>415</v>
@@ -67861,7 +67861,7 @@
         <v>0</v>
       </c>
       <c r="N351" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O351" s="15" t="s">
         <v>415</v>
@@ -68061,7 +68061,7 @@
         <v>0</v>
       </c>
       <c r="N352" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O352" s="15" t="s">
         <v>415</v>
@@ -68249,7 +68249,7 @@
         <v>2</v>
       </c>
       <c r="N353" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O353" s="15" t="s">
         <v>415</v>
@@ -68441,7 +68441,7 @@
         <v>2</v>
       </c>
       <c r="N354" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O354" s="15" t="s">
         <v>247</v>
@@ -68483,7 +68483,7 @@
         <v>181</v>
       </c>
       <c r="AB354" s="14" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="AC354" s="14" t="s">
         <v>134</v>
@@ -68637,7 +68637,7 @@
         <v>5</v>
       </c>
       <c r="N355" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O355" s="15" t="s">
         <v>415</v>
@@ -68843,7 +68843,7 @@
         <v>3</v>
       </c>
       <c r="N356" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O356" s="15" t="s">
         <v>247</v>
@@ -69069,7 +69069,7 @@
         <v>4</v>
       </c>
       <c r="N357" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O357" s="15" t="s">
         <v>415</v>
@@ -69111,7 +69111,7 @@
         <v>145</v>
       </c>
       <c r="AB357" s="14" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AC357" s="14" t="s">
         <v>285</v>
@@ -69263,7 +69263,7 @@
         <v>2</v>
       </c>
       <c r="N358" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O358" s="15" t="s">
         <v>415</v>
@@ -69311,7 +69311,7 @@
         <v>587</v>
       </c>
       <c r="AD358" s="14" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="AE358" s="14" t="s">
         <v>181</v>
@@ -69465,7 +69465,7 @@
         <v>2</v>
       </c>
       <c r="N359" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O359" s="15" t="s">
         <v>244</v>
@@ -69657,7 +69657,7 @@
         <v>1</v>
       </c>
       <c r="N360" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O360" s="15" t="s">
         <v>415</v>
@@ -69865,7 +69865,7 @@
         <v>3</v>
       </c>
       <c r="N361" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O361" s="15" t="s">
         <v>244</v>
@@ -70073,7 +70073,7 @@
         <v>0</v>
       </c>
       <c r="N362" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O362" s="15" t="s">
         <v>415</v>
@@ -70121,7 +70121,7 @@
         <v>591</v>
       </c>
       <c r="AD362" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="AE362" s="14" t="s">
         <v>106</v>
@@ -70283,7 +70283,7 @@
         <v>8</v>
       </c>
       <c r="N363" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O363" s="15" t="s">
         <v>244</v>
@@ -70325,7 +70325,7 @@
         <v>181</v>
       </c>
       <c r="AB363" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="AC363" s="14" t="s">
         <v>145</v>
@@ -70334,7 +70334,7 @@
         <v>138</v>
       </c>
       <c r="AE363" s="14" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="AF363" s="14"/>
       <c r="AG363" s="14"/>
@@ -70477,7 +70477,7 @@
         <v>4</v>
       </c>
       <c r="N364" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
       <c r="O364" s="15" t="s">
         <v>415</v>
@@ -70522,7 +70522,7 @@
         <v>108</v>
       </c>
       <c r="AC364" s="14" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="AD364" s="14" t="s">
         <v>106</v>
@@ -70667,7 +70667,7 @@
         <v>1</v>
       </c>
       <c r="N365" s="19" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="O365" s="15" t="s">
         <v>415</v>
@@ -70883,7 +70883,7 @@
         <v>595</v>
       </c>
       <c r="N366" s="19" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="O366" s="15" t="s">
         <v>415</v>

</xml_diff>